<commit_message>
feat(export): update course outline excel template and multi-column budget layout
</commit_message>
<xml_diff>
--- a/app/Excel/ATA-F-HD-005-Couse Outline.xlsx
+++ b/app/Excel/ATA-F-HD-005-Couse Outline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trainee\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ECE0244-6E60-4F48-B5C2-A8934D305137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EC3D662-0E37-4FD9-9997-7ECE7000C6FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{BC99A250-FEBB-43EA-840D-941C3158CE7C}"/>
   </bookViews>
@@ -650,7 +650,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
@@ -772,18 +772,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="188" fontId="5" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="188" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -833,20 +821,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -857,8 +833,14 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1065,7 +1047,7 @@
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1600">
+          <a:endParaRPr lang="th-TH" sz="1600">
             <a:solidFill>
               <a:sysClr val="windowText" lastClr="000000"/>
             </a:solidFill>
@@ -1180,6 +1162,132 @@
         </xdr:spPr>
       </xdr:pic>
     </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>175260</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FB15E0F8-65D3-0F89-CA9B-49B09ED11896}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="83820" y="8732520"/>
+          <a:ext cx="4229100" cy="3253740"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="th-TH" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>251460</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>259080</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="TextBox 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1CA39CA5-1936-5FDB-6528-F8F5CEAE683C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4389120" y="3962400"/>
+          <a:ext cx="4861560" cy="1188720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="th-TH" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -1486,6 +1594,195 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>129540</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="TextBox 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2C7F8BD-9A4B-D5B6-8481-7187334A0F07}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4404360" y="2682240"/>
+          <a:ext cx="4792980" cy="944880"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="th-TH" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>144780</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="TextBox 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{442C1EDC-75E6-5831-4CC5-51B31CA29F7C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="91440" y="8732520"/>
+          <a:ext cx="4191000" cy="3215640"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="th-TH" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>251460</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>129540</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>266700</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="TextBox 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0F1DC388-E8FF-3FFF-D376-9A2B3603FEDA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4389120" y="4008120"/>
+          <a:ext cx="4808220" cy="1150620"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:endParaRPr lang="th-TH" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1512,6 +1809,28 @@
       <sheetName val="A"/>
       <sheetName val="DATA_STD_VC_EXPORT1"/>
       <sheetName val="Cash_Gen_1"/>
+      <sheetName val="DATA_STD_VC_EXPORT2"/>
+      <sheetName val="Cash_Gen_2"/>
+      <sheetName val="DATA_STD_VC_EXPORT3"/>
+      <sheetName val="Cash_Gen_3"/>
+      <sheetName val="DATA_STD_VC_EXPORT4"/>
+      <sheetName val="Cash_Gen_4"/>
+      <sheetName val="DATA_STD_VC_EXPORT5"/>
+      <sheetName val="Cash_Gen_5"/>
+      <sheetName val="DATA_STD_VC_EXPORT6"/>
+      <sheetName val="Cash_Gen_6"/>
+      <sheetName val="PS"/>
+      <sheetName val="CODE"/>
+      <sheetName val="61B (J)"/>
+      <sheetName val="X61B (E)"/>
+      <sheetName val="DATA_STD_VC_EXPORT7"/>
+      <sheetName val="Cash_Gen_7"/>
+      <sheetName val="61B_(J)"/>
+      <sheetName val="X61B_(E)"/>
+      <sheetName val="DATA_STD_VC_EXPORT8"/>
+      <sheetName val="Cash_Gen_8"/>
+      <sheetName val="61B_(J)1"/>
+      <sheetName val="X61B_(E)1"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -1533,6 +1852,28 @@
       <sheetData sheetId="16" refreshError="1"/>
       <sheetData sheetId="17"/>
       <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
+      <sheetData sheetId="25"/>
+      <sheetData sheetId="26"/>
+      <sheetData sheetId="27"/>
+      <sheetData sheetId="28"/>
+      <sheetData sheetId="29" refreshError="1"/>
+      <sheetData sheetId="30" refreshError="1"/>
+      <sheetData sheetId="31" refreshError="1"/>
+      <sheetData sheetId="32" refreshError="1"/>
+      <sheetData sheetId="33"/>
+      <sheetData sheetId="34"/>
+      <sheetData sheetId="35"/>
+      <sheetData sheetId="36"/>
+      <sheetData sheetId="37"/>
+      <sheetData sheetId="38"/>
+      <sheetData sheetId="39"/>
+      <sheetData sheetId="40"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -2937,26 +3278,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="8.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="65"/>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
-      <c r="N1" s="89"/>
-      <c r="O1" s="90"/>
+      <c r="A1" s="59"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
+      <c r="N1" s="83"/>
+      <c r="O1" s="84"/>
       <c r="P1" s="3"/>
       <c r="Q1" s="3"/>
     </row>
     <row r="2" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A2" s="71"/>
+      <c r="A2" s="65"/>
       <c r="B2" s="48"/>
       <c r="C2" s="48"/>
       <c r="D2" s="48"/>
@@ -2967,21 +3308,21 @@
       <c r="I2" s="49"/>
       <c r="J2" s="49"/>
       <c r="K2" s="49"/>
-      <c r="L2" s="68" t="s">
+      <c r="L2" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="69" t="s">
+      <c r="M2" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="N2" s="70" t="s">
+      <c r="N2" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="87"/>
+      <c r="O2" s="81"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
     </row>
     <row r="3" spans="1:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A3" s="71"/>
+      <c r="A3" s="65"/>
       <c r="B3" s="48"/>
       <c r="C3" s="48"/>
       <c r="D3" s="48"/>
@@ -2995,12 +3336,12 @@
       <c r="L3" s="43"/>
       <c r="M3" s="41"/>
       <c r="N3" s="45"/>
-      <c r="O3" s="72"/>
+      <c r="O3" s="66"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A4" s="71"/>
+      <c r="A4" s="65"/>
       <c r="B4" s="48"/>
       <c r="C4" s="48"/>
       <c r="D4" s="48"/>
@@ -3014,12 +3355,12 @@
       <c r="L4" s="44"/>
       <c r="M4" s="42"/>
       <c r="N4" s="46"/>
-      <c r="O4" s="72"/>
+      <c r="O4" s="66"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A5" s="71"/>
+      <c r="A5" s="65"/>
       <c r="B5" s="48"/>
       <c r="C5" s="48"/>
       <c r="D5" s="48"/>
@@ -3039,12 +3380,12 @@
       <c r="N5" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="O5" s="72"/>
+      <c r="O5" s="66"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
     </row>
     <row r="6" spans="1:17" ht="25.2" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="A6" s="71"/>
+      <c r="A6" s="65"/>
       <c r="B6" s="48"/>
       <c r="C6" s="48"/>
       <c r="D6" s="48"/>
@@ -3064,33 +3405,33 @@
       <c r="N6" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="O6" s="72"/>
+      <c r="O6" s="66"/>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="36" customHeight="1" thickTop="1" x14ac:dyDescent="0.8">
-      <c r="A7" s="71"/>
-      <c r="B7" s="97" t="s">
+      <c r="A7" s="65"/>
+      <c r="B7" s="87" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="97"/>
-      <c r="D7" s="97"/>
-      <c r="E7" s="97"/>
-      <c r="F7" s="97"/>
-      <c r="G7" s="97"/>
-      <c r="H7" s="97"/>
-      <c r="I7" s="97"/>
-      <c r="J7" s="97"/>
-      <c r="K7" s="97"/>
-      <c r="L7" s="97"/>
-      <c r="M7" s="97"/>
-      <c r="N7" s="97"/>
-      <c r="O7" s="73"/>
+      <c r="C7" s="87"/>
+      <c r="D7" s="87"/>
+      <c r="E7" s="87"/>
+      <c r="F7" s="87"/>
+      <c r="G7" s="87"/>
+      <c r="H7" s="87"/>
+      <c r="I7" s="87"/>
+      <c r="J7" s="87"/>
+      <c r="K7" s="87"/>
+      <c r="L7" s="87"/>
+      <c r="M7" s="87"/>
+      <c r="N7" s="87"/>
+      <c r="O7" s="67"/>
       <c r="P7" s="5"/>
       <c r="Q7" s="5"/>
     </row>
     <row r="8" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A8" s="71"/>
+      <c r="A8" s="65"/>
       <c r="B8" s="49"/>
       <c r="C8" s="49"/>
       <c r="D8" s="49"/>
@@ -3104,12 +3445,12 @@
       <c r="L8" s="49"/>
       <c r="M8" s="49"/>
       <c r="N8" s="49"/>
-      <c r="O8" s="74"/>
+      <c r="O8" s="68"/>
       <c r="P8" s="5"/>
       <c r="Q8" s="5"/>
     </row>
     <row r="9" spans="1:17" ht="27.6" x14ac:dyDescent="0.8">
-      <c r="A9" s="71"/>
+      <c r="A9" s="65"/>
       <c r="B9" s="50" t="s">
         <v>1</v>
       </c>
@@ -3127,10 +3468,10 @@
       <c r="L9" s="50"/>
       <c r="M9" s="50"/>
       <c r="N9" s="50"/>
-      <c r="O9" s="75"/>
+      <c r="O9" s="69"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A10" s="71"/>
+      <c r="A10" s="65"/>
       <c r="B10" s="47"/>
       <c r="C10" s="47"/>
       <c r="D10" s="47"/>
@@ -3140,16 +3481,16 @@
       <c r="H10" s="47"/>
       <c r="I10" s="47"/>
       <c r="J10" s="47"/>
-      <c r="K10" s="96"/>
-      <c r="L10" s="96"/>
-      <c r="M10" s="96"/>
-      <c r="N10" s="96"/>
-      <c r="O10" s="76"/>
+      <c r="K10" s="93"/>
+      <c r="L10" s="93"/>
+      <c r="M10" s="93"/>
+      <c r="N10" s="93"/>
+      <c r="O10" s="70"/>
       <c r="P10" s="7"/>
       <c r="Q10" s="7"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A11" s="71"/>
+      <c r="A11" s="65"/>
       <c r="B11" s="48"/>
       <c r="C11" s="48"/>
       <c r="D11" s="48"/>
@@ -3159,16 +3500,16 @@
       <c r="H11" s="48"/>
       <c r="I11" s="48"/>
       <c r="J11" s="47"/>
-      <c r="K11" s="96"/>
-      <c r="L11" s="96"/>
-      <c r="M11" s="96"/>
-      <c r="N11" s="96"/>
-      <c r="O11" s="76"/>
+      <c r="K11" s="93"/>
+      <c r="L11" s="93"/>
+      <c r="M11" s="93"/>
+      <c r="N11" s="93"/>
+      <c r="O11" s="70"/>
       <c r="P11" s="7"/>
       <c r="Q11" s="7"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A12" s="71"/>
+      <c r="A12" s="65"/>
       <c r="B12" s="48"/>
       <c r="C12" s="48"/>
       <c r="D12" s="48"/>
@@ -3178,16 +3519,16 @@
       <c r="H12" s="48"/>
       <c r="I12" s="48"/>
       <c r="J12" s="47"/>
-      <c r="K12" s="96"/>
-      <c r="L12" s="96"/>
-      <c r="M12" s="96"/>
-      <c r="N12" s="96"/>
-      <c r="O12" s="76"/>
+      <c r="K12" s="93"/>
+      <c r="L12" s="93"/>
+      <c r="M12" s="93"/>
+      <c r="N12" s="93"/>
+      <c r="O12" s="70"/>
       <c r="P12" s="7"/>
       <c r="Q12" s="7"/>
     </row>
     <row r="13" spans="1:17" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A13" s="71"/>
+      <c r="A13" s="65"/>
       <c r="B13" s="48"/>
       <c r="C13" s="48"/>
       <c r="D13" s="48"/>
@@ -3203,10 +3544,10 @@
       <c r="L13" s="52"/>
       <c r="M13" s="52"/>
       <c r="N13" s="52"/>
-      <c r="O13" s="75"/>
+      <c r="O13" s="69"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A14" s="71"/>
+      <c r="A14" s="65"/>
       <c r="B14" s="48"/>
       <c r="C14" s="48"/>
       <c r="D14" s="48"/>
@@ -3216,16 +3557,16 @@
       <c r="H14" s="48"/>
       <c r="I14" s="48"/>
       <c r="J14" s="47"/>
-      <c r="K14" s="96"/>
-      <c r="L14" s="96"/>
-      <c r="M14" s="96"/>
-      <c r="N14" s="96"/>
-      <c r="O14" s="77"/>
+      <c r="K14" s="93"/>
+      <c r="L14" s="93"/>
+      <c r="M14" s="93"/>
+      <c r="N14" s="93"/>
+      <c r="O14" s="71"/>
       <c r="P14" s="6"/>
       <c r="Q14" s="6"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A15" s="71"/>
+      <c r="A15" s="65"/>
       <c r="B15" s="48"/>
       <c r="C15" s="48"/>
       <c r="D15" s="48"/>
@@ -3235,16 +3576,16 @@
       <c r="H15" s="48"/>
       <c r="I15" s="48"/>
       <c r="J15" s="47"/>
-      <c r="K15" s="96"/>
-      <c r="L15" s="96"/>
-      <c r="M15" s="96"/>
-      <c r="N15" s="96"/>
-      <c r="O15" s="78"/>
+      <c r="K15" s="93"/>
+      <c r="L15" s="93"/>
+      <c r="M15" s="93"/>
+      <c r="N15" s="93"/>
+      <c r="O15" s="72"/>
       <c r="P15" s="8"/>
       <c r="Q15" s="8"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A16" s="71"/>
+      <c r="A16" s="65"/>
       <c r="B16" s="53"/>
       <c r="C16" s="48"/>
       <c r="D16" s="48"/>
@@ -3254,16 +3595,16 @@
       <c r="H16" s="48"/>
       <c r="I16" s="48"/>
       <c r="J16" s="47"/>
-      <c r="K16" s="96"/>
-      <c r="L16" s="96"/>
-      <c r="M16" s="96"/>
-      <c r="N16" s="96"/>
-      <c r="O16" s="76"/>
+      <c r="K16" s="93"/>
+      <c r="L16" s="93"/>
+      <c r="M16" s="93"/>
+      <c r="N16" s="93"/>
+      <c r="O16" s="70"/>
       <c r="P16" s="7"/>
       <c r="Q16" s="7"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A17" s="71"/>
+      <c r="A17" s="65"/>
       <c r="B17" s="53"/>
       <c r="C17" s="48"/>
       <c r="D17" s="48"/>
@@ -3273,14 +3614,14 @@
       <c r="H17" s="48"/>
       <c r="I17" s="48"/>
       <c r="J17" s="47"/>
-      <c r="K17" s="96"/>
-      <c r="L17" s="96"/>
-      <c r="M17" s="96"/>
-      <c r="N17" s="96"/>
-      <c r="O17" s="75"/>
+      <c r="K17" s="93"/>
+      <c r="L17" s="93"/>
+      <c r="M17" s="93"/>
+      <c r="N17" s="93"/>
+      <c r="O17" s="69"/>
     </row>
     <row r="18" spans="1:19" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A18" s="71"/>
+      <c r="A18" s="65"/>
       <c r="B18" s="50" t="s">
         <v>4</v>
       </c>
@@ -3298,10 +3639,10 @@
       <c r="L18" s="52"/>
       <c r="M18" s="52"/>
       <c r="N18" s="52"/>
-      <c r="O18" s="75"/>
+      <c r="O18" s="69"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A19" s="71"/>
+      <c r="A19" s="65"/>
       <c r="B19" s="48"/>
       <c r="C19" s="48"/>
       <c r="D19" s="48"/>
@@ -3317,12 +3658,12 @@
       <c r="L19" s="48"/>
       <c r="M19" s="48"/>
       <c r="N19" s="48"/>
-      <c r="O19" s="79"/>
+      <c r="O19" s="73"/>
       <c r="P19" s="10"/>
       <c r="Q19" s="9"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A20" s="71"/>
+      <c r="A20" s="65"/>
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
       <c r="D20" s="48"/>
@@ -3338,12 +3679,12 @@
       <c r="L20" s="48"/>
       <c r="M20" s="48"/>
       <c r="N20" s="47"/>
-      <c r="O20" s="75"/>
+      <c r="O20" s="69"/>
       <c r="P20" s="9"/>
       <c r="Q20" s="2"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A21" s="71"/>
+      <c r="A21" s="65"/>
       <c r="B21" s="53"/>
       <c r="C21" s="48"/>
       <c r="D21" s="48"/>
@@ -3359,12 +3700,12 @@
       <c r="L21" s="48"/>
       <c r="M21" s="48"/>
       <c r="N21" s="56"/>
-      <c r="O21" s="80"/>
+      <c r="O21" s="74"/>
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A22" s="71"/>
+      <c r="A22" s="65"/>
       <c r="B22" s="47"/>
       <c r="C22" s="47"/>
       <c r="D22" s="47"/>
@@ -3378,10 +3719,10 @@
       <c r="L22" s="47"/>
       <c r="M22" s="47"/>
       <c r="N22" s="47"/>
-      <c r="O22" s="75"/>
+      <c r="O22" s="69"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A23" s="71"/>
+      <c r="A23" s="65"/>
       <c r="B23" s="47"/>
       <c r="C23" s="58"/>
       <c r="D23" s="58"/>
@@ -3395,10 +3736,10 @@
       <c r="L23" s="47"/>
       <c r="M23" s="47"/>
       <c r="N23" s="47"/>
-      <c r="O23" s="75"/>
+      <c r="O23" s="69"/>
     </row>
     <row r="24" spans="1:19" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A24" s="71"/>
+      <c r="A24" s="65"/>
       <c r="B24" s="47"/>
       <c r="C24" s="47"/>
       <c r="D24" s="47"/>
@@ -3414,10 +3755,10 @@
       <c r="L24" s="52"/>
       <c r="M24" s="52"/>
       <c r="N24" s="52"/>
-      <c r="O24" s="75"/>
+      <c r="O24" s="69"/>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A25" s="71"/>
+      <c r="A25" s="65"/>
       <c r="B25" s="47"/>
       <c r="C25" s="47"/>
       <c r="D25" s="47"/>
@@ -3427,14 +3768,14 @@
       <c r="H25" s="47"/>
       <c r="I25" s="47"/>
       <c r="J25" s="47"/>
-      <c r="K25" s="96"/>
-      <c r="L25" s="96"/>
-      <c r="M25" s="96"/>
-      <c r="N25" s="96"/>
-      <c r="O25" s="75"/>
+      <c r="K25" s="93"/>
+      <c r="L25" s="93"/>
+      <c r="M25" s="93"/>
+      <c r="N25" s="93"/>
+      <c r="O25" s="69"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A26" s="71"/>
+      <c r="A26" s="65"/>
       <c r="B26" s="47"/>
       <c r="C26" s="47"/>
       <c r="D26" s="47"/>
@@ -3444,14 +3785,14 @@
       <c r="H26" s="47"/>
       <c r="I26" s="47"/>
       <c r="J26" s="47"/>
-      <c r="K26" s="96"/>
-      <c r="L26" s="96"/>
-      <c r="M26" s="96"/>
-      <c r="N26" s="96"/>
-      <c r="O26" s="75"/>
+      <c r="K26" s="93"/>
+      <c r="L26" s="93"/>
+      <c r="M26" s="93"/>
+      <c r="N26" s="93"/>
+      <c r="O26" s="69"/>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A27" s="71"/>
+      <c r="A27" s="65"/>
       <c r="B27" s="47"/>
       <c r="C27" s="47"/>
       <c r="D27" s="47"/>
@@ -3461,14 +3802,14 @@
       <c r="H27" s="47"/>
       <c r="I27" s="47"/>
       <c r="J27" s="47"/>
-      <c r="K27" s="96"/>
-      <c r="L27" s="96"/>
-      <c r="M27" s="96"/>
-      <c r="N27" s="96"/>
-      <c r="O27" s="75"/>
+      <c r="K27" s="93"/>
+      <c r="L27" s="93"/>
+      <c r="M27" s="93"/>
+      <c r="N27" s="93"/>
+      <c r="O27" s="69"/>
     </row>
     <row r="28" spans="1:19" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A28" s="71"/>
+      <c r="A28" s="65"/>
       <c r="B28" s="50" t="s">
         <v>10</v>
       </c>
@@ -3480,225 +3821,225 @@
       <c r="H28" s="52"/>
       <c r="I28" s="52"/>
       <c r="J28" s="47"/>
-      <c r="K28" s="96"/>
-      <c r="L28" s="96"/>
-      <c r="M28" s="96"/>
-      <c r="N28" s="96"/>
-      <c r="O28" s="75"/>
+      <c r="K28" s="93"/>
+      <c r="L28" s="93"/>
+      <c r="M28" s="93"/>
+      <c r="N28" s="93"/>
+      <c r="O28" s="69"/>
       <c r="P28" s="5"/>
       <c r="Q28" s="5"/>
       <c r="S28" s="13"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A29" s="71"/>
-      <c r="B29" s="96"/>
-      <c r="C29" s="96"/>
-      <c r="D29" s="96"/>
-      <c r="E29" s="96"/>
-      <c r="F29" s="96"/>
-      <c r="G29" s="96"/>
-      <c r="H29" s="96"/>
-      <c r="I29" s="96"/>
+      <c r="A29" s="65"/>
+      <c r="B29" s="93"/>
+      <c r="C29" s="93"/>
+      <c r="D29" s="93"/>
+      <c r="E29" s="93"/>
+      <c r="F29" s="93"/>
+      <c r="G29" s="93"/>
+      <c r="H29" s="93"/>
+      <c r="I29" s="93"/>
       <c r="J29" s="47"/>
-      <c r="K29" s="96"/>
-      <c r="L29" s="96"/>
-      <c r="M29" s="96"/>
-      <c r="N29" s="96"/>
-      <c r="O29" s="72"/>
+      <c r="K29" s="93"/>
+      <c r="L29" s="93"/>
+      <c r="M29" s="93"/>
+      <c r="N29" s="93"/>
+      <c r="O29" s="66"/>
       <c r="P29" s="2"/>
       <c r="Q29" s="2"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A30" s="71"/>
-      <c r="B30" s="96"/>
-      <c r="C30" s="96"/>
-      <c r="D30" s="96"/>
-      <c r="E30" s="96"/>
-      <c r="F30" s="96"/>
-      <c r="G30" s="96"/>
-      <c r="H30" s="96"/>
-      <c r="I30" s="96"/>
+      <c r="A30" s="65"/>
+      <c r="B30" s="93"/>
+      <c r="C30" s="93"/>
+      <c r="D30" s="93"/>
+      <c r="E30" s="93"/>
+      <c r="F30" s="93"/>
+      <c r="G30" s="93"/>
+      <c r="H30" s="93"/>
+      <c r="I30" s="93"/>
       <c r="J30" s="47"/>
-      <c r="K30" s="96"/>
-      <c r="L30" s="96"/>
-      <c r="M30" s="96"/>
-      <c r="N30" s="96"/>
-      <c r="O30" s="72"/>
+      <c r="K30" s="93"/>
+      <c r="L30" s="93"/>
+      <c r="M30" s="93"/>
+      <c r="N30" s="93"/>
+      <c r="O30" s="66"/>
       <c r="P30" s="2"/>
       <c r="Q30" s="15"/>
     </row>
-    <row r="31" spans="1:19" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A31" s="71"/>
-      <c r="B31" s="96"/>
-      <c r="C31" s="96"/>
-      <c r="D31" s="96"/>
-      <c r="E31" s="96"/>
-      <c r="F31" s="96"/>
-      <c r="G31" s="96"/>
-      <c r="H31" s="96"/>
-      <c r="I31" s="96"/>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.7">
+      <c r="A31" s="65"/>
+      <c r="B31" s="93"/>
+      <c r="C31" s="93"/>
+      <c r="D31" s="93"/>
+      <c r="E31" s="93"/>
+      <c r="F31" s="93"/>
+      <c r="G31" s="93"/>
+      <c r="H31" s="93"/>
+      <c r="I31" s="93"/>
       <c r="J31" s="47"/>
-      <c r="K31" s="50" t="s">
+      <c r="K31" s="92"/>
+      <c r="L31" s="92"/>
+      <c r="M31" s="92"/>
+      <c r="N31" s="92"/>
+      <c r="O31" s="75"/>
+      <c r="P31" s="16"/>
+      <c r="Q31" s="16"/>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.7">
+      <c r="A32" s="65"/>
+      <c r="B32" s="93"/>
+      <c r="C32" s="93"/>
+      <c r="D32" s="93"/>
+      <c r="E32" s="93"/>
+      <c r="F32" s="93"/>
+      <c r="G32" s="93"/>
+      <c r="H32" s="93"/>
+      <c r="I32" s="93"/>
+      <c r="J32" s="47"/>
+      <c r="K32" s="92"/>
+      <c r="L32" s="92"/>
+      <c r="M32" s="92"/>
+      <c r="N32" s="92"/>
+      <c r="O32" s="75"/>
+      <c r="P32" s="16"/>
+      <c r="Q32" s="16"/>
+    </row>
+    <row r="33" spans="1:27" ht="26.4" x14ac:dyDescent="0.7">
+      <c r="A33" s="65"/>
+      <c r="B33" s="93"/>
+      <c r="C33" s="93"/>
+      <c r="D33" s="93"/>
+      <c r="E33" s="93"/>
+      <c r="F33" s="93"/>
+      <c r="G33" s="93"/>
+      <c r="H33" s="93"/>
+      <c r="I33" s="93"/>
+      <c r="J33" s="47"/>
+      <c r="K33" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="L31" s="52"/>
-      <c r="M31" s="52"/>
-      <c r="N31" s="52"/>
-      <c r="O31" s="81"/>
-      <c r="P31" s="16"/>
-      <c r="Q31" s="16"/>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A32" s="71"/>
-      <c r="B32" s="96"/>
-      <c r="C32" s="96"/>
-      <c r="D32" s="96"/>
-      <c r="E32" s="96"/>
-      <c r="F32" s="96"/>
-      <c r="G32" s="96"/>
-      <c r="H32" s="96"/>
-      <c r="I32" s="96"/>
-      <c r="J32" s="47"/>
-      <c r="K32" s="96"/>
-      <c r="L32" s="96"/>
-      <c r="M32" s="96"/>
-      <c r="N32" s="96"/>
-      <c r="O32" s="81"/>
-      <c r="P32" s="16"/>
-      <c r="Q32" s="16"/>
-    </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A33" s="71"/>
-      <c r="B33" s="96"/>
-      <c r="C33" s="96"/>
-      <c r="D33" s="96"/>
-      <c r="E33" s="96"/>
-      <c r="F33" s="96"/>
-      <c r="G33" s="96"/>
-      <c r="H33" s="96"/>
-      <c r="I33" s="96"/>
-      <c r="J33" s="47"/>
-      <c r="K33" s="96"/>
-      <c r="L33" s="96"/>
-      <c r="M33" s="96"/>
-      <c r="N33" s="96"/>
-      <c r="O33" s="81"/>
+      <c r="L33" s="52"/>
+      <c r="M33" s="52"/>
+      <c r="N33" s="52"/>
+      <c r="O33" s="75"/>
       <c r="P33" s="16"/>
       <c r="Q33" s="16"/>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A34" s="71"/>
-      <c r="B34" s="100"/>
-      <c r="C34" s="100"/>
-      <c r="D34" s="100"/>
-      <c r="E34" s="100"/>
-      <c r="F34" s="100"/>
-      <c r="G34" s="100"/>
-      <c r="H34" s="100"/>
-      <c r="I34" s="100"/>
+      <c r="A34" s="65"/>
+      <c r="B34" s="92"/>
+      <c r="C34" s="92"/>
+      <c r="D34" s="92"/>
+      <c r="E34" s="92"/>
+      <c r="F34" s="92"/>
+      <c r="G34" s="92"/>
+      <c r="H34" s="92"/>
+      <c r="I34" s="92"/>
       <c r="J34" s="47"/>
-      <c r="K34" s="96"/>
-      <c r="L34" s="96"/>
-      <c r="M34" s="96"/>
-      <c r="N34" s="96"/>
-      <c r="O34" s="81"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="93"/>
+      <c r="M34" s="93"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="75"/>
       <c r="P34" s="16"/>
       <c r="Q34" s="16"/>
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A35" s="71"/>
-      <c r="B35" s="96"/>
-      <c r="C35" s="96"/>
-      <c r="D35" s="96"/>
-      <c r="E35" s="96"/>
-      <c r="F35" s="96"/>
-      <c r="G35" s="96"/>
-      <c r="H35" s="96"/>
-      <c r="I35" s="96"/>
+      <c r="A35" s="65"/>
+      <c r="B35" s="93"/>
+      <c r="C35" s="93"/>
+      <c r="D35" s="93"/>
+      <c r="E35" s="93"/>
+      <c r="F35" s="93"/>
+      <c r="G35" s="93"/>
+      <c r="H35" s="93"/>
+      <c r="I35" s="93"/>
       <c r="J35" s="47"/>
-      <c r="K35" s="96"/>
-      <c r="L35" s="96"/>
-      <c r="M35" s="96"/>
-      <c r="N35" s="96"/>
-      <c r="O35" s="72"/>
+      <c r="K35" s="93"/>
+      <c r="L35" s="93"/>
+      <c r="M35" s="93"/>
+      <c r="N35" s="93"/>
+      <c r="O35" s="66"/>
       <c r="P35" s="2"/>
       <c r="Q35" s="2"/>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A36" s="71"/>
-      <c r="B36" s="95"/>
-      <c r="C36" s="95"/>
-      <c r="D36" s="95"/>
-      <c r="E36" s="95"/>
-      <c r="F36" s="95"/>
-      <c r="G36" s="95"/>
-      <c r="H36" s="95"/>
-      <c r="I36" s="95"/>
+      <c r="A36" s="65"/>
+      <c r="B36" s="86"/>
+      <c r="C36" s="86"/>
+      <c r="D36" s="86"/>
+      <c r="E36" s="86"/>
+      <c r="F36" s="86"/>
+      <c r="G36" s="86"/>
+      <c r="H36" s="86"/>
+      <c r="I36" s="86"/>
       <c r="J36" s="47"/>
-      <c r="K36" s="96"/>
-      <c r="L36" s="96"/>
-      <c r="M36" s="96"/>
-      <c r="N36" s="96"/>
-      <c r="O36" s="72"/>
+      <c r="K36" s="93"/>
+      <c r="L36" s="93"/>
+      <c r="M36" s="93"/>
+      <c r="N36" s="93"/>
+      <c r="O36" s="66"/>
       <c r="P36" s="2"/>
       <c r="Q36" s="2"/>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A37" s="71"/>
-      <c r="B37" s="95"/>
-      <c r="C37" s="95"/>
-      <c r="D37" s="95"/>
-      <c r="E37" s="95"/>
-      <c r="F37" s="95"/>
-      <c r="G37" s="95"/>
-      <c r="H37" s="95"/>
-      <c r="I37" s="95"/>
+      <c r="A37" s="65"/>
+      <c r="B37" s="86"/>
+      <c r="C37" s="86"/>
+      <c r="D37" s="86"/>
+      <c r="E37" s="86"/>
+      <c r="F37" s="86"/>
+      <c r="G37" s="86"/>
+      <c r="H37" s="86"/>
+      <c r="I37" s="86"/>
       <c r="J37" s="47"/>
-      <c r="K37" s="96"/>
-      <c r="L37" s="96"/>
-      <c r="M37" s="96"/>
-      <c r="N37" s="96"/>
-      <c r="O37" s="72"/>
+      <c r="K37" s="93"/>
+      <c r="L37" s="93"/>
+      <c r="M37" s="93"/>
+      <c r="N37" s="93"/>
+      <c r="O37" s="66"/>
       <c r="P37" s="2"/>
       <c r="Q37" s="2"/>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A38" s="71"/>
-      <c r="B38" s="96"/>
-      <c r="C38" s="96"/>
-      <c r="D38" s="96"/>
-      <c r="E38" s="96"/>
-      <c r="F38" s="96"/>
-      <c r="G38" s="96"/>
-      <c r="H38" s="96"/>
-      <c r="I38" s="96"/>
+      <c r="A38" s="65"/>
+      <c r="B38" s="93"/>
+      <c r="C38" s="93"/>
+      <c r="D38" s="93"/>
+      <c r="E38" s="93"/>
+      <c r="F38" s="93"/>
+      <c r="G38" s="93"/>
+      <c r="H38" s="93"/>
+      <c r="I38" s="93"/>
       <c r="J38" s="47"/>
-      <c r="K38" s="96"/>
-      <c r="L38" s="96"/>
-      <c r="M38" s="96"/>
-      <c r="N38" s="96"/>
-      <c r="O38" s="75"/>
+      <c r="K38" s="93"/>
+      <c r="L38" s="93"/>
+      <c r="M38" s="93"/>
+      <c r="N38" s="93"/>
+      <c r="O38" s="69"/>
       <c r="T38" s="2"/>
       <c r="U38" s="2"/>
     </row>
     <row r="39" spans="1:27" ht="32.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="A39" s="82" t="s">
+      <c r="A39" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="B39" s="83"/>
-      <c r="C39" s="84"/>
-      <c r="D39" s="84"/>
-      <c r="E39" s="84"/>
-      <c r="F39" s="84"/>
-      <c r="G39" s="84"/>
-      <c r="H39" s="84"/>
-      <c r="I39" s="84"/>
-      <c r="J39" s="85"/>
-      <c r="K39" s="96"/>
-      <c r="L39" s="96"/>
-      <c r="M39" s="96"/>
-      <c r="N39" s="96"/>
-      <c r="O39" s="86"/>
+      <c r="B39" s="77"/>
+      <c r="C39" s="78"/>
+      <c r="D39" s="78"/>
+      <c r="E39" s="78"/>
+      <c r="F39" s="78"/>
+      <c r="G39" s="78"/>
+      <c r="H39" s="78"/>
+      <c r="I39" s="78"/>
+      <c r="J39" s="79"/>
+      <c r="K39" s="93"/>
+      <c r="L39" s="93"/>
+      <c r="M39" s="93"/>
+      <c r="N39" s="93"/>
+      <c r="O39" s="80"/>
       <c r="T39" s="11"/>
       <c r="U39" s="11"/>
     </row>
@@ -3712,7 +4053,7 @@
     <row r="41" spans="1:27" x14ac:dyDescent="0.7">
       <c r="B41" s="18"/>
       <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
+      <c r="K41" s="48"/>
       <c r="L41" s="2"/>
       <c r="M41" s="14"/>
     </row>
@@ -3803,13 +4144,13 @@
     </row>
     <row r="49" spans="2:27" x14ac:dyDescent="0.7">
       <c r="B49" s="12"/>
-      <c r="C49" s="99"/>
-      <c r="D49" s="99"/>
-      <c r="E49" s="99"/>
-      <c r="F49" s="99"/>
-      <c r="G49" s="99"/>
-      <c r="H49" s="99"/>
-      <c r="I49" s="99"/>
+      <c r="C49" s="89"/>
+      <c r="D49" s="89"/>
+      <c r="E49" s="89"/>
+      <c r="F49" s="89"/>
+      <c r="G49" s="89"/>
+      <c r="H49" s="89"/>
+      <c r="I49" s="89"/>
       <c r="J49" s="23"/>
       <c r="S49" s="12"/>
       <c r="T49" s="8"/>
@@ -3842,13 +4183,13 @@
     </row>
     <row r="51" spans="2:27" x14ac:dyDescent="0.7">
       <c r="B51" s="26"/>
-      <c r="C51" s="98"/>
-      <c r="D51" s="98"/>
-      <c r="E51" s="98"/>
-      <c r="F51" s="98"/>
-      <c r="G51" s="98"/>
-      <c r="H51" s="98"/>
-      <c r="I51" s="98"/>
+      <c r="C51" s="88"/>
+      <c r="D51" s="88"/>
+      <c r="E51" s="88"/>
+      <c r="F51" s="88"/>
+      <c r="G51" s="88"/>
+      <c r="H51" s="88"/>
+      <c r="I51" s="88"/>
       <c r="S51" s="12"/>
       <c r="T51" s="27"/>
       <c r="U51" s="27"/>
@@ -3915,13 +4256,13 @@
       <c r="AA54" s="27"/>
     </row>
     <row r="55" spans="2:27" x14ac:dyDescent="0.7">
-      <c r="C55" s="98"/>
-      <c r="D55" s="98"/>
-      <c r="E55" s="98"/>
-      <c r="F55" s="98"/>
-      <c r="G55" s="98"/>
-      <c r="H55" s="98"/>
-      <c r="I55" s="98"/>
+      <c r="C55" s="88"/>
+      <c r="D55" s="88"/>
+      <c r="E55" s="88"/>
+      <c r="F55" s="88"/>
+      <c r="G55" s="88"/>
+      <c r="H55" s="88"/>
+      <c r="I55" s="88"/>
       <c r="S55" s="12"/>
       <c r="T55" s="2"/>
       <c r="U55" s="2"/>
@@ -4004,40 +4345,11 @@
       <c r="Z62" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="K30:N30"/>
-    <mergeCell ref="K32:N32"/>
-    <mergeCell ref="K33:N33"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="K34:N34"/>
-    <mergeCell ref="K35:N35"/>
+  <mergeCells count="4">
     <mergeCell ref="C55:I55"/>
     <mergeCell ref="C49:I49"/>
     <mergeCell ref="C51:I51"/>
-    <mergeCell ref="K36:N36"/>
-    <mergeCell ref="K37:N37"/>
-    <mergeCell ref="K38:N38"/>
-    <mergeCell ref="K39:N39"/>
-    <mergeCell ref="B34:I34"/>
-    <mergeCell ref="B35:I35"/>
     <mergeCell ref="B7:N7"/>
-    <mergeCell ref="K14:N14"/>
-    <mergeCell ref="K15:N15"/>
-    <mergeCell ref="K16:N16"/>
-    <mergeCell ref="K17:N17"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="K11:N11"/>
-    <mergeCell ref="K12:N12"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="K27:N27"/>
-    <mergeCell ref="K28:N28"/>
-    <mergeCell ref="K29:N29"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0"/>
@@ -5146,26 +5458,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="8.4" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="A1" s="65"/>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="89"/>
-      <c r="M1" s="89"/>
-      <c r="N1" s="89"/>
-      <c r="O1" s="90"/>
+      <c r="A1" s="59"/>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
+      <c r="N1" s="83"/>
+      <c r="O1" s="84"/>
       <c r="P1" s="3"/>
       <c r="Q1" s="3"/>
     </row>
     <row r="2" spans="1:17" ht="24.75" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A2" s="71"/>
+      <c r="A2" s="65"/>
       <c r="B2" s="48"/>
       <c r="C2" s="48"/>
       <c r="D2" s="48"/>
@@ -5176,21 +5488,21 @@
       <c r="I2" s="49"/>
       <c r="J2" s="49"/>
       <c r="K2" s="49"/>
-      <c r="L2" s="68" t="s">
+      <c r="L2" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="69" t="s">
+      <c r="M2" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="N2" s="70" t="s">
+      <c r="N2" s="64" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="87"/>
+      <c r="O2" s="81"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
     </row>
     <row r="3" spans="1:17" ht="26.25" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A3" s="71"/>
+      <c r="A3" s="65"/>
       <c r="B3" s="48"/>
       <c r="C3" s="48"/>
       <c r="D3" s="48"/>
@@ -5204,12 +5516,12 @@
       <c r="L3" s="43"/>
       <c r="M3" s="41"/>
       <c r="N3" s="45"/>
-      <c r="O3" s="72"/>
+      <c r="O3" s="66"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A4" s="71"/>
+      <c r="A4" s="65"/>
       <c r="B4" s="48"/>
       <c r="C4" s="48"/>
       <c r="D4" s="48"/>
@@ -5223,12 +5535,12 @@
       <c r="L4" s="44"/>
       <c r="M4" s="42"/>
       <c r="N4" s="46"/>
-      <c r="O4" s="72"/>
+      <c r="O4" s="66"/>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A5" s="71"/>
+      <c r="A5" s="65"/>
       <c r="B5" s="48"/>
       <c r="C5" s="48"/>
       <c r="D5" s="48"/>
@@ -5248,12 +5560,12 @@
       <c r="N5" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="O5" s="72"/>
+      <c r="O5" s="66"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
     </row>
     <row r="6" spans="1:17" ht="25.2" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="A6" s="71"/>
+      <c r="A6" s="65"/>
       <c r="B6" s="48"/>
       <c r="C6" s="48"/>
       <c r="D6" s="48"/>
@@ -5273,33 +5585,33 @@
       <c r="N6" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="O6" s="72"/>
+      <c r="O6" s="66"/>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
     </row>
     <row r="7" spans="1:17" ht="36" customHeight="1" thickTop="1" x14ac:dyDescent="0.8">
-      <c r="A7" s="71"/>
-      <c r="B7" s="97" t="s">
+      <c r="A7" s="65"/>
+      <c r="B7" s="87" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="97"/>
-      <c r="D7" s="97"/>
-      <c r="E7" s="97"/>
-      <c r="F7" s="97"/>
-      <c r="G7" s="97"/>
-      <c r="H7" s="97"/>
-      <c r="I7" s="97"/>
-      <c r="J7" s="97"/>
-      <c r="K7" s="97"/>
-      <c r="L7" s="97"/>
-      <c r="M7" s="97"/>
-      <c r="N7" s="97"/>
-      <c r="O7" s="73"/>
+      <c r="C7" s="87"/>
+      <c r="D7" s="87"/>
+      <c r="E7" s="87"/>
+      <c r="F7" s="87"/>
+      <c r="G7" s="87"/>
+      <c r="H7" s="87"/>
+      <c r="I7" s="87"/>
+      <c r="J7" s="87"/>
+      <c r="K7" s="87"/>
+      <c r="L7" s="87"/>
+      <c r="M7" s="87"/>
+      <c r="N7" s="87"/>
+      <c r="O7" s="67"/>
       <c r="P7" s="5"/>
       <c r="Q7" s="5"/>
     </row>
     <row r="8" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A8" s="71"/>
+      <c r="A8" s="65"/>
       <c r="B8" s="49"/>
       <c r="C8" s="49"/>
       <c r="D8" s="49"/>
@@ -5313,12 +5625,12 @@
       <c r="L8" s="49"/>
       <c r="M8" s="49"/>
       <c r="N8" s="49"/>
-      <c r="O8" s="74"/>
+      <c r="O8" s="68"/>
       <c r="P8" s="5"/>
       <c r="Q8" s="5"/>
     </row>
     <row r="9" spans="1:17" ht="27.6" x14ac:dyDescent="0.8">
-      <c r="A9" s="71"/>
+      <c r="A9" s="65"/>
       <c r="B9" s="50" t="s">
         <v>13</v>
       </c>
@@ -5336,10 +5648,10 @@
       <c r="L9" s="50"/>
       <c r="M9" s="50"/>
       <c r="N9" s="50"/>
-      <c r="O9" s="75"/>
+      <c r="O9" s="69"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A10" s="71"/>
+      <c r="A10" s="65"/>
       <c r="B10" s="47"/>
       <c r="C10" s="47"/>
       <c r="D10" s="47"/>
@@ -5349,16 +5661,16 @@
       <c r="H10" s="47"/>
       <c r="I10" s="47"/>
       <c r="J10" s="47"/>
-      <c r="K10" s="96"/>
-      <c r="L10" s="96"/>
-      <c r="M10" s="96"/>
-      <c r="N10" s="96"/>
-      <c r="O10" s="76"/>
+      <c r="K10" s="93"/>
+      <c r="L10" s="93"/>
+      <c r="M10" s="93"/>
+      <c r="N10" s="93"/>
+      <c r="O10" s="70"/>
       <c r="P10" s="7"/>
       <c r="Q10" s="7"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A11" s="71"/>
+      <c r="A11" s="65"/>
       <c r="B11" s="48"/>
       <c r="C11" s="48"/>
       <c r="D11" s="48"/>
@@ -5368,16 +5680,16 @@
       <c r="H11" s="48"/>
       <c r="I11" s="48"/>
       <c r="J11" s="47"/>
-      <c r="K11" s="96"/>
-      <c r="L11" s="96"/>
-      <c r="M11" s="96"/>
-      <c r="N11" s="96"/>
-      <c r="O11" s="76"/>
+      <c r="K11" s="93"/>
+      <c r="L11" s="93"/>
+      <c r="M11" s="93"/>
+      <c r="N11" s="93"/>
+      <c r="O11" s="70"/>
       <c r="P11" s="7"/>
       <c r="Q11" s="7"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A12" s="71"/>
+      <c r="A12" s="65"/>
       <c r="B12" s="48"/>
       <c r="C12" s="48"/>
       <c r="D12" s="48"/>
@@ -5387,16 +5699,16 @@
       <c r="H12" s="48"/>
       <c r="I12" s="48"/>
       <c r="J12" s="47"/>
-      <c r="K12" s="96"/>
-      <c r="L12" s="96"/>
-      <c r="M12" s="96"/>
-      <c r="N12" s="96"/>
-      <c r="O12" s="76"/>
+      <c r="K12" s="93"/>
+      <c r="L12" s="93"/>
+      <c r="M12" s="93"/>
+      <c r="N12" s="93"/>
+      <c r="O12" s="70"/>
       <c r="P12" s="7"/>
       <c r="Q12" s="7"/>
     </row>
     <row r="13" spans="1:17" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A13" s="71"/>
+      <c r="A13" s="65"/>
       <c r="B13" s="48"/>
       <c r="C13" s="48"/>
       <c r="D13" s="48"/>
@@ -5412,10 +5724,10 @@
       <c r="L13" s="52"/>
       <c r="M13" s="52"/>
       <c r="N13" s="52"/>
-      <c r="O13" s="75"/>
+      <c r="O13" s="69"/>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A14" s="71"/>
+      <c r="A14" s="65"/>
       <c r="B14" s="48"/>
       <c r="C14" s="48"/>
       <c r="D14" s="48"/>
@@ -5425,16 +5737,15 @@
       <c r="H14" s="48"/>
       <c r="I14" s="48"/>
       <c r="J14" s="47"/>
-      <c r="K14" s="96"/>
-      <c r="L14" s="96"/>
-      <c r="M14" s="96"/>
-      <c r="N14" s="96"/>
-      <c r="O14" s="77"/>
+      <c r="K14" s="93"/>
+      <c r="M14" s="93"/>
+      <c r="N14" s="93"/>
+      <c r="O14" s="71"/>
       <c r="P14" s="6"/>
       <c r="Q14" s="6"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A15" s="71"/>
+      <c r="A15" s="65"/>
       <c r="B15" s="48"/>
       <c r="C15" s="48"/>
       <c r="D15" s="48"/>
@@ -5444,16 +5755,13 @@
       <c r="H15" s="48"/>
       <c r="I15" s="48"/>
       <c r="J15" s="47"/>
-      <c r="K15" s="96"/>
-      <c r="L15" s="96"/>
-      <c r="M15" s="96"/>
-      <c r="N15" s="96"/>
-      <c r="O15" s="78"/>
+      <c r="K15" s="94"/>
+      <c r="O15" s="72"/>
       <c r="P15" s="8"/>
       <c r="Q15" s="8"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.7">
-      <c r="A16" s="71"/>
+      <c r="A16" s="65"/>
       <c r="B16" s="53"/>
       <c r="C16" s="48"/>
       <c r="D16" s="48"/>
@@ -5463,16 +5771,16 @@
       <c r="H16" s="48"/>
       <c r="I16" s="48"/>
       <c r="J16" s="47"/>
-      <c r="K16" s="96"/>
-      <c r="L16" s="96"/>
-      <c r="M16" s="96"/>
-      <c r="N16" s="96"/>
-      <c r="O16" s="76"/>
+      <c r="K16" s="93"/>
+      <c r="L16" s="93"/>
+      <c r="M16" s="93"/>
+      <c r="N16" s="93"/>
+      <c r="O16" s="70"/>
       <c r="P16" s="7"/>
       <c r="Q16" s="7"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A17" s="71"/>
+      <c r="A17" s="65"/>
       <c r="B17" s="53"/>
       <c r="C17" s="48"/>
       <c r="D17" s="48"/>
@@ -5482,14 +5790,14 @@
       <c r="H17" s="48"/>
       <c r="I17" s="48"/>
       <c r="J17" s="47"/>
-      <c r="K17" s="91"/>
-      <c r="L17" s="91"/>
-      <c r="M17" s="91"/>
-      <c r="N17" s="91"/>
-      <c r="O17" s="75"/>
+      <c r="K17" s="85"/>
+      <c r="L17" s="85"/>
+      <c r="M17" s="85"/>
+      <c r="N17" s="85"/>
+      <c r="O17" s="69"/>
     </row>
     <row r="18" spans="1:19" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A18" s="71"/>
+      <c r="A18" s="65"/>
       <c r="B18" s="50" t="s">
         <v>16</v>
       </c>
@@ -5507,10 +5815,10 @@
       <c r="L18" s="52"/>
       <c r="M18" s="52"/>
       <c r="N18" s="52"/>
-      <c r="O18" s="75"/>
+      <c r="O18" s="69"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A19" s="71"/>
+      <c r="A19" s="65"/>
       <c r="B19" s="48"/>
       <c r="C19" s="48"/>
       <c r="D19" s="48"/>
@@ -5526,12 +5834,12 @@
       <c r="L19" s="48"/>
       <c r="M19" s="48"/>
       <c r="N19" s="48"/>
-      <c r="O19" s="79"/>
+      <c r="O19" s="73"/>
       <c r="P19" s="10"/>
       <c r="Q19" s="9"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A20" s="71"/>
+      <c r="A20" s="65"/>
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
       <c r="D20" s="48"/>
@@ -5547,12 +5855,12 @@
       <c r="L20" s="48"/>
       <c r="M20" s="48"/>
       <c r="N20" s="47"/>
-      <c r="O20" s="75"/>
+      <c r="O20" s="69"/>
       <c r="P20" s="9"/>
       <c r="Q20" s="2"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A21" s="71"/>
+      <c r="A21" s="65"/>
       <c r="B21" s="53"/>
       <c r="C21" s="48"/>
       <c r="D21" s="48"/>
@@ -5568,12 +5876,12 @@
       <c r="L21" s="48"/>
       <c r="M21" s="48"/>
       <c r="N21" s="56"/>
-      <c r="O21" s="80"/>
+      <c r="O21" s="74"/>
       <c r="P21" s="2"/>
       <c r="Q21" s="2"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A22" s="71"/>
+      <c r="A22" s="65"/>
       <c r="B22" s="47"/>
       <c r="C22" s="47"/>
       <c r="D22" s="47"/>
@@ -5587,10 +5895,10 @@
       <c r="L22" s="47"/>
       <c r="M22" s="47"/>
       <c r="N22" s="47"/>
-      <c r="O22" s="75"/>
+      <c r="O22" s="69"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A23" s="71"/>
+      <c r="A23" s="65"/>
       <c r="B23" s="47"/>
       <c r="C23" s="58"/>
       <c r="D23" s="58"/>
@@ -5604,10 +5912,10 @@
       <c r="L23" s="47"/>
       <c r="M23" s="47"/>
       <c r="N23" s="47"/>
-      <c r="O23" s="75"/>
+      <c r="O23" s="69"/>
     </row>
     <row r="24" spans="1:19" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A24" s="71"/>
+      <c r="A24" s="65"/>
       <c r="B24" s="47"/>
       <c r="C24" s="47"/>
       <c r="D24" s="47"/>
@@ -5623,10 +5931,10 @@
       <c r="L24" s="52"/>
       <c r="M24" s="52"/>
       <c r="N24" s="52"/>
-      <c r="O24" s="75"/>
+      <c r="O24" s="69"/>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A25" s="71"/>
+      <c r="A25" s="65"/>
       <c r="B25" s="47"/>
       <c r="C25" s="47"/>
       <c r="D25" s="47"/>
@@ -5636,14 +5944,14 @@
       <c r="H25" s="47"/>
       <c r="I25" s="47"/>
       <c r="J25" s="47"/>
-      <c r="K25" s="59"/>
-      <c r="L25" s="48"/>
-      <c r="M25" s="60"/>
-      <c r="N25" s="61"/>
-      <c r="O25" s="75"/>
+      <c r="K25" s="91"/>
+      <c r="L25" s="91"/>
+      <c r="M25" s="91"/>
+      <c r="N25" s="91"/>
+      <c r="O25" s="69"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A26" s="71"/>
+      <c r="A26" s="65"/>
       <c r="B26" s="47"/>
       <c r="C26" s="47"/>
       <c r="D26" s="47"/>
@@ -5653,14 +5961,14 @@
       <c r="H26" s="47"/>
       <c r="I26" s="47"/>
       <c r="J26" s="47"/>
-      <c r="K26" s="59"/>
-      <c r="L26" s="48"/>
-      <c r="M26" s="60"/>
-      <c r="N26" s="61"/>
-      <c r="O26" s="75"/>
+      <c r="K26" s="91"/>
+      <c r="L26" s="91"/>
+      <c r="M26" s="91"/>
+      <c r="N26" s="91"/>
+      <c r="O26" s="69"/>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A27" s="71"/>
+      <c r="A27" s="65"/>
       <c r="B27" s="47"/>
       <c r="C27" s="47"/>
       <c r="D27" s="47"/>
@@ -5670,14 +5978,14 @@
       <c r="H27" s="47"/>
       <c r="I27" s="47"/>
       <c r="J27" s="47"/>
-      <c r="K27" s="59"/>
-      <c r="L27" s="48"/>
-      <c r="M27" s="60"/>
-      <c r="N27" s="61"/>
-      <c r="O27" s="75"/>
+      <c r="K27" s="91"/>
+      <c r="L27" s="91"/>
+      <c r="M27" s="91"/>
+      <c r="N27" s="91"/>
+      <c r="O27" s="69"/>
     </row>
     <row r="28" spans="1:19" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A28" s="71"/>
+      <c r="A28" s="65"/>
       <c r="B28" s="50" t="s">
         <v>19</v>
       </c>
@@ -5689,225 +5997,225 @@
       <c r="H28" s="52"/>
       <c r="I28" s="52"/>
       <c r="J28" s="47"/>
-      <c r="K28" s="48"/>
-      <c r="L28" s="62"/>
-      <c r="M28" s="63"/>
-      <c r="N28" s="61"/>
-      <c r="O28" s="75"/>
+      <c r="K28" s="90"/>
+      <c r="L28" s="90"/>
+      <c r="M28" s="90"/>
+      <c r="N28" s="90"/>
+      <c r="O28" s="69"/>
       <c r="P28" s="5"/>
       <c r="Q28" s="5"/>
       <c r="S28" s="13"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A29" s="71"/>
-      <c r="B29" s="96"/>
-      <c r="C29" s="96"/>
-      <c r="D29" s="96"/>
-      <c r="E29" s="96"/>
-      <c r="F29" s="96"/>
-      <c r="G29" s="96"/>
-      <c r="H29" s="96"/>
-      <c r="I29" s="96"/>
+      <c r="A29" s="65"/>
+      <c r="B29" s="93"/>
+      <c r="C29" s="93"/>
+      <c r="D29" s="93"/>
+      <c r="E29" s="93"/>
+      <c r="F29" s="93"/>
+      <c r="G29" s="93"/>
+      <c r="H29" s="93"/>
+      <c r="I29" s="93"/>
       <c r="J29" s="47"/>
-      <c r="K29" s="48"/>
-      <c r="L29" s="64"/>
-      <c r="M29" s="48"/>
-      <c r="N29" s="47"/>
-      <c r="O29" s="72"/>
+      <c r="K29" s="90"/>
+      <c r="L29" s="90"/>
+      <c r="M29" s="90"/>
+      <c r="N29" s="90"/>
+      <c r="O29" s="66"/>
       <c r="P29" s="2"/>
       <c r="Q29" s="2"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A30" s="71"/>
-      <c r="B30" s="96"/>
-      <c r="C30" s="96"/>
-      <c r="D30" s="96"/>
-      <c r="E30" s="96"/>
-      <c r="F30" s="96"/>
-      <c r="G30" s="96"/>
-      <c r="H30" s="96"/>
-      <c r="I30" s="96"/>
+      <c r="A30" s="65"/>
+      <c r="B30" s="93"/>
+      <c r="C30" s="93"/>
+      <c r="D30" s="93"/>
+      <c r="E30" s="93"/>
+      <c r="F30" s="93"/>
+      <c r="G30" s="93"/>
+      <c r="H30" s="93"/>
+      <c r="I30" s="93"/>
       <c r="J30" s="47"/>
-      <c r="K30" s="48"/>
-      <c r="L30" s="64"/>
-      <c r="M30" s="48"/>
-      <c r="N30" s="47"/>
-      <c r="O30" s="72"/>
+      <c r="K30" s="90"/>
+      <c r="L30" s="90"/>
+      <c r="M30" s="90"/>
+      <c r="N30" s="90"/>
+      <c r="O30" s="66"/>
       <c r="P30" s="2"/>
       <c r="Q30" s="15"/>
     </row>
-    <row r="31" spans="1:19" ht="26.4" x14ac:dyDescent="0.7">
-      <c r="A31" s="71"/>
-      <c r="B31" s="96"/>
-      <c r="C31" s="96"/>
-      <c r="D31" s="96"/>
-      <c r="E31" s="96"/>
-      <c r="F31" s="96"/>
-      <c r="G31" s="96"/>
-      <c r="H31" s="96"/>
-      <c r="I31" s="96"/>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.7">
+      <c r="A31" s="65"/>
+      <c r="B31" s="93"/>
+      <c r="C31" s="93"/>
+      <c r="D31" s="93"/>
+      <c r="E31" s="93"/>
+      <c r="F31" s="93"/>
+      <c r="G31" s="93"/>
+      <c r="H31" s="93"/>
+      <c r="I31" s="93"/>
       <c r="J31" s="47"/>
-      <c r="K31" s="50" t="s">
+      <c r="K31" s="92"/>
+      <c r="L31" s="92"/>
+      <c r="M31" s="92"/>
+      <c r="N31" s="92"/>
+      <c r="O31" s="75"/>
+      <c r="P31" s="16"/>
+      <c r="Q31" s="16"/>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.7">
+      <c r="A32" s="65"/>
+      <c r="B32" s="93"/>
+      <c r="C32" s="93"/>
+      <c r="D32" s="93"/>
+      <c r="E32" s="93"/>
+      <c r="F32" s="93"/>
+      <c r="G32" s="93"/>
+      <c r="H32" s="93"/>
+      <c r="I32" s="93"/>
+      <c r="J32" s="47"/>
+      <c r="K32" s="90"/>
+      <c r="L32" s="90"/>
+      <c r="M32" s="90"/>
+      <c r="N32" s="90"/>
+      <c r="O32" s="75"/>
+      <c r="P32" s="16"/>
+      <c r="Q32" s="16"/>
+    </row>
+    <row r="33" spans="1:27" ht="26.4" x14ac:dyDescent="0.7">
+      <c r="A33" s="65"/>
+      <c r="B33" s="93"/>
+      <c r="C33" s="93"/>
+      <c r="D33" s="93"/>
+      <c r="E33" s="93"/>
+      <c r="F33" s="93"/>
+      <c r="G33" s="93"/>
+      <c r="H33" s="93"/>
+      <c r="I33" s="93"/>
+      <c r="J33" s="47"/>
+      <c r="K33" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="L31" s="52"/>
-      <c r="M31" s="52"/>
-      <c r="N31" s="52"/>
-      <c r="O31" s="81"/>
-      <c r="P31" s="16"/>
-      <c r="Q31" s="16"/>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.7">
-      <c r="A32" s="71"/>
-      <c r="B32" s="96"/>
-      <c r="C32" s="96"/>
-      <c r="D32" s="96"/>
-      <c r="E32" s="96"/>
-      <c r="F32" s="96"/>
-      <c r="G32" s="96"/>
-      <c r="H32" s="96"/>
-      <c r="I32" s="96"/>
-      <c r="J32" s="47"/>
-      <c r="K32" s="96"/>
-      <c r="L32" s="96"/>
-      <c r="M32" s="96"/>
-      <c r="N32" s="96"/>
-      <c r="O32" s="81"/>
-      <c r="P32" s="16"/>
-      <c r="Q32" s="16"/>
-    </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A33" s="71"/>
-      <c r="B33" s="96"/>
-      <c r="C33" s="96"/>
-      <c r="D33" s="96"/>
-      <c r="E33" s="96"/>
-      <c r="F33" s="96"/>
-      <c r="G33" s="96"/>
-      <c r="H33" s="96"/>
-      <c r="I33" s="96"/>
-      <c r="J33" s="47"/>
-      <c r="K33" s="96"/>
-      <c r="L33" s="96"/>
-      <c r="M33" s="96"/>
-      <c r="N33" s="96"/>
-      <c r="O33" s="81"/>
+      <c r="L33" s="52"/>
+      <c r="M33" s="52"/>
+      <c r="N33" s="52"/>
+      <c r="O33" s="75"/>
       <c r="P33" s="16"/>
       <c r="Q33" s="16"/>
     </row>
     <row r="34" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A34" s="71"/>
-      <c r="B34" s="96"/>
-      <c r="C34" s="96"/>
-      <c r="D34" s="96"/>
-      <c r="E34" s="96"/>
-      <c r="F34" s="96"/>
-      <c r="G34" s="96"/>
-      <c r="H34" s="96"/>
-      <c r="I34" s="96"/>
+      <c r="A34" s="65"/>
+      <c r="B34" s="93"/>
+      <c r="C34" s="93"/>
+      <c r="D34" s="93"/>
+      <c r="E34" s="93"/>
+      <c r="F34" s="93"/>
+      <c r="G34" s="93"/>
+      <c r="H34" s="93"/>
+      <c r="I34" s="93"/>
       <c r="J34" s="47"/>
-      <c r="K34" s="96"/>
-      <c r="L34" s="96"/>
-      <c r="M34" s="96"/>
-      <c r="N34" s="96"/>
-      <c r="O34" s="81"/>
+      <c r="K34" s="93"/>
+      <c r="L34" s="93"/>
+      <c r="M34" s="93"/>
+      <c r="N34" s="93"/>
+      <c r="O34" s="75"/>
       <c r="P34" s="16"/>
       <c r="Q34" s="16"/>
     </row>
     <row r="35" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A35" s="71"/>
-      <c r="B35" s="96"/>
-      <c r="C35" s="96"/>
-      <c r="D35" s="96"/>
-      <c r="E35" s="96"/>
-      <c r="F35" s="96"/>
-      <c r="G35" s="96"/>
-      <c r="H35" s="96"/>
-      <c r="I35" s="96"/>
+      <c r="A35" s="65"/>
+      <c r="B35" s="93"/>
+      <c r="C35" s="93"/>
+      <c r="D35" s="93"/>
+      <c r="E35" s="93"/>
+      <c r="F35" s="93"/>
+      <c r="G35" s="93"/>
+      <c r="H35" s="93"/>
+      <c r="I35" s="93"/>
       <c r="J35" s="47"/>
-      <c r="K35" s="56"/>
-      <c r="L35" s="56"/>
-      <c r="M35" s="56"/>
-      <c r="N35" s="91"/>
-      <c r="O35" s="72"/>
+      <c r="K35" s="90"/>
+      <c r="L35" s="90"/>
+      <c r="M35" s="90"/>
+      <c r="N35" s="90"/>
+      <c r="O35" s="66"/>
       <c r="P35" s="2"/>
       <c r="Q35" s="2"/>
     </row>
     <row r="36" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A36" s="71"/>
-      <c r="B36" s="96"/>
-      <c r="C36" s="96"/>
-      <c r="D36" s="96"/>
-      <c r="E36" s="96"/>
-      <c r="F36" s="96"/>
-      <c r="G36" s="96"/>
-      <c r="H36" s="96"/>
-      <c r="I36" s="96"/>
+      <c r="A36" s="65"/>
+      <c r="B36" s="93"/>
+      <c r="C36" s="93"/>
+      <c r="D36" s="93"/>
+      <c r="E36" s="93"/>
+      <c r="F36" s="93"/>
+      <c r="G36" s="93"/>
+      <c r="H36" s="93"/>
+      <c r="I36" s="93"/>
       <c r="J36" s="47"/>
-      <c r="K36" s="92"/>
-      <c r="L36" s="92"/>
-      <c r="M36" s="92"/>
-      <c r="N36" s="92"/>
-      <c r="O36" s="72"/>
+      <c r="K36" s="90"/>
+      <c r="L36" s="90"/>
+      <c r="M36" s="90"/>
+      <c r="N36" s="90"/>
+      <c r="O36" s="66"/>
       <c r="P36" s="2"/>
       <c r="Q36" s="2"/>
     </row>
     <row r="37" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A37" s="71"/>
-      <c r="B37" s="96"/>
-      <c r="C37" s="96"/>
-      <c r="D37" s="96"/>
-      <c r="E37" s="96"/>
-      <c r="F37" s="96"/>
-      <c r="G37" s="96"/>
-      <c r="H37" s="96"/>
-      <c r="I37" s="96"/>
+      <c r="A37" s="65"/>
+      <c r="B37" s="93"/>
+      <c r="C37" s="93"/>
+      <c r="D37" s="93"/>
+      <c r="E37" s="93"/>
+      <c r="F37" s="93"/>
+      <c r="G37" s="93"/>
+      <c r="H37" s="93"/>
+      <c r="I37" s="93"/>
       <c r="J37" s="47"/>
-      <c r="K37" s="92"/>
-      <c r="L37" s="92"/>
-      <c r="M37" s="56"/>
-      <c r="N37" s="92"/>
-      <c r="O37" s="72"/>
+      <c r="K37" s="90"/>
+      <c r="L37" s="90"/>
+      <c r="M37" s="90"/>
+      <c r="N37" s="90"/>
+      <c r="O37" s="66"/>
       <c r="P37" s="2"/>
       <c r="Q37" s="2"/>
     </row>
     <row r="38" spans="1:27" x14ac:dyDescent="0.7">
-      <c r="A38" s="71"/>
-      <c r="B38" s="96"/>
-      <c r="C38" s="96"/>
-      <c r="D38" s="96"/>
-      <c r="E38" s="96"/>
-      <c r="F38" s="96"/>
-      <c r="G38" s="96"/>
-      <c r="H38" s="96"/>
-      <c r="I38" s="96"/>
+      <c r="A38" s="65"/>
+      <c r="B38" s="93"/>
+      <c r="C38" s="93"/>
+      <c r="D38" s="93"/>
+      <c r="E38" s="93"/>
+      <c r="F38" s="93"/>
+      <c r="G38" s="93"/>
+      <c r="H38" s="93"/>
+      <c r="I38" s="93"/>
       <c r="J38" s="47"/>
-      <c r="K38" s="92"/>
-      <c r="L38" s="92"/>
-      <c r="M38" s="56"/>
-      <c r="N38" s="92"/>
-      <c r="O38" s="75"/>
+      <c r="K38" s="90"/>
+      <c r="L38" s="90"/>
+      <c r="M38" s="90"/>
+      <c r="N38" s="90"/>
+      <c r="O38" s="69"/>
       <c r="T38" s="2"/>
       <c r="U38" s="2"/>
     </row>
     <row r="39" spans="1:27" ht="32.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="A39" s="82" t="s">
+      <c r="A39" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="B39" s="83"/>
-      <c r="C39" s="84"/>
-      <c r="D39" s="84"/>
-      <c r="E39" s="84"/>
-      <c r="F39" s="84"/>
-      <c r="G39" s="84"/>
-      <c r="H39" s="84"/>
-      <c r="I39" s="84"/>
-      <c r="J39" s="85"/>
-      <c r="K39" s="93"/>
-      <c r="L39" s="93"/>
-      <c r="M39" s="93"/>
-      <c r="N39" s="94"/>
-      <c r="O39" s="86"/>
+      <c r="B39" s="77"/>
+      <c r="C39" s="78"/>
+      <c r="D39" s="78"/>
+      <c r="E39" s="78"/>
+      <c r="F39" s="78"/>
+      <c r="G39" s="78"/>
+      <c r="H39" s="78"/>
+      <c r="I39" s="78"/>
+      <c r="J39" s="79"/>
+      <c r="K39" s="90"/>
+      <c r="L39" s="90"/>
+      <c r="M39" s="90"/>
+      <c r="N39" s="90"/>
+      <c r="O39" s="80"/>
       <c r="T39" s="11"/>
       <c r="U39" s="11"/>
     </row>
@@ -6012,13 +6320,13 @@
     </row>
     <row r="49" spans="2:27" x14ac:dyDescent="0.7">
       <c r="B49" s="12"/>
-      <c r="C49" s="99"/>
-      <c r="D49" s="99"/>
-      <c r="E49" s="99"/>
-      <c r="F49" s="99"/>
-      <c r="G49" s="99"/>
-      <c r="H49" s="99"/>
-      <c r="I49" s="99"/>
+      <c r="C49" s="89"/>
+      <c r="D49" s="89"/>
+      <c r="E49" s="89"/>
+      <c r="F49" s="89"/>
+      <c r="G49" s="89"/>
+      <c r="H49" s="89"/>
+      <c r="I49" s="89"/>
       <c r="J49" s="23"/>
       <c r="S49" s="12"/>
       <c r="T49" s="8"/>
@@ -6051,13 +6359,13 @@
     </row>
     <row r="51" spans="2:27" x14ac:dyDescent="0.7">
       <c r="B51" s="26"/>
-      <c r="C51" s="98"/>
-      <c r="D51" s="98"/>
-      <c r="E51" s="98"/>
-      <c r="F51" s="98"/>
-      <c r="G51" s="98"/>
-      <c r="H51" s="98"/>
-      <c r="I51" s="98"/>
+      <c r="C51" s="88"/>
+      <c r="D51" s="88"/>
+      <c r="E51" s="88"/>
+      <c r="F51" s="88"/>
+      <c r="G51" s="88"/>
+      <c r="H51" s="88"/>
+      <c r="I51" s="88"/>
       <c r="S51" s="12"/>
       <c r="T51" s="27"/>
       <c r="U51" s="27"/>
@@ -6124,13 +6432,13 @@
       <c r="AA54" s="27"/>
     </row>
     <row r="55" spans="2:27" x14ac:dyDescent="0.7">
-      <c r="C55" s="98"/>
-      <c r="D55" s="98"/>
-      <c r="E55" s="98"/>
-      <c r="F55" s="98"/>
-      <c r="G55" s="98"/>
-      <c r="H55" s="98"/>
-      <c r="I55" s="98"/>
+      <c r="C55" s="88"/>
+      <c r="D55" s="88"/>
+      <c r="E55" s="88"/>
+      <c r="F55" s="88"/>
+      <c r="G55" s="88"/>
+      <c r="H55" s="88"/>
+      <c r="I55" s="88"/>
       <c r="S55" s="12"/>
       <c r="T55" s="2"/>
       <c r="U55" s="2"/>
@@ -6213,30 +6521,11 @@
       <c r="Z62" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="B37:I37"/>
-    <mergeCell ref="B36:I36"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="K32:N32"/>
-    <mergeCell ref="K33:N33"/>
-    <mergeCell ref="K34:N34"/>
-    <mergeCell ref="B34:I34"/>
+  <mergeCells count="4">
     <mergeCell ref="B7:N7"/>
     <mergeCell ref="C49:I49"/>
     <mergeCell ref="C51:I51"/>
     <mergeCell ref="C55:I55"/>
-    <mergeCell ref="K10:N10"/>
-    <mergeCell ref="K11:N11"/>
-    <mergeCell ref="K12:N12"/>
-    <mergeCell ref="K14:N14"/>
-    <mergeCell ref="K15:N15"/>
-    <mergeCell ref="K16:N16"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B35:I35"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0"/>

</xml_diff>